<commit_message>
Rename RIConstructionActivity to RIColumnConstruction in dictionary bindings
Follows the schema rename. Five workbooks edited and regenerated: riInstallationMethod,
terminationOutcome, groutLevelCorrectiveAction, grout_inj_properties, correctiveAction.

Seven sourceElementXpath bindings repointed from //diggs:RIConstructionActivity/... to
//diggs:RIColumnConstruction/..., plus prose references in six dictionary and entry
descriptions.

Workbook-first as always; the generated XML was produced by xlsx_2_xml, not hand-edited.
Every regenerated file was word-diffed to confirm the only change is the rename.

The quote-escaping artifact fired again on gr_inj_properties.xml, unescaping &quot; in a
pre-existing entry this rename never touched, and was re-escaped per the settled default.
That file's diff went from 2 changed lines to 1 as a result.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/groutLevelCorrectiveAction.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/groutLevelCorrectiveAction.xlsx
@@ -985,7 +985,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Codes for the corrective action taken where in-progress grout-level monitoring found the grout level in a rigid inclusion column had dropped below the expected level - an 'uncovered column' condition indicating grout loss into the surrounding ground (V2 Installation row 31). Used for the value of diggs:RIConstructionActivityType/groutLevelCorrectiveAction.</t>
+          <t>Codes for the corrective action taken where in-progress grout-level monitoring found the grout level in a rigid inclusion column had dropped below the expected level - an 'uncovered column' condition indicating grout loss into the surrounding ground (V2 Installation row 31). Used for the value of diggs:RIColumnConstructionType/groutLevelCorrectiveAction.</t>
         </is>
       </c>
     </row>
@@ -1594,7 +1594,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>//diggs:RIConstructionActivity/diggs:groutLevelCorrectiveAction</t>
+          <t>//diggs:RIColumnConstruction/diggs:groutLevelCorrectiveAction</t>
         </is>
       </c>
     </row>
@@ -1610,7 +1610,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>//diggs:RIConstructionActivity/diggs:groutLevelCorrectiveAction</t>
+          <t>//diggs:RIColumnConstruction/diggs:groutLevelCorrectiveAction</t>
         </is>
       </c>
     </row>
@@ -1626,7 +1626,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>//diggs:RIConstructionActivity/diggs:groutLevelCorrectiveAction</t>
+          <t>//diggs:RIColumnConstruction/diggs:groutLevelCorrectiveAction</t>
         </is>
       </c>
     </row>

</xml_diff>